<commit_message>
lci modelling and lcia notebooks
</commit_message>
<xml_diff>
--- a/premise/data/additional_inventories/lci-hydrogen-transport.xlsx
+++ b/premise/data/additional_inventories/lci-hydrogen-transport.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ac145674\coding_projects\premise_h2-distribution\premise\data\additional_inventories\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A06CC5E4-059D-47C7-B7EA-C88B21E09681}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6CBAFE06-043C-4FF3-9C2D-B8E35A7EAB79}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8652" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8655" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="hydrogen-transport" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="919" uniqueCount="216">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="926" uniqueCount="217">
   <si>
     <t>Database</t>
   </si>
@@ -670,6 +670,9 @@
   </si>
   <si>
     <t>NH3+MDO</t>
+  </si>
+  <si>
+    <t>electricity needed for the processes and compression</t>
   </si>
 </sst>
 </file>
@@ -1118,24 +1121,24 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L217"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
+  <dimension ref="A1:L218"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="82.6640625" customWidth="1"/>
-    <col min="2" max="2" width="9.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="82.7109375" customWidth="1"/>
+    <col min="2" max="2" width="9.85546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="23" customWidth="1"/>
-    <col min="4" max="4" width="13.6640625" customWidth="1"/>
-    <col min="5" max="5" width="17.109375" customWidth="1"/>
-    <col min="6" max="6" width="16.109375" customWidth="1"/>
-    <col min="7" max="7" width="85.44140625" customWidth="1"/>
-    <col min="8" max="8" width="25.44140625" customWidth="1"/>
-    <col min="11" max="11" width="13.33203125" customWidth="1"/>
-    <col min="12" max="12" width="43.88671875" customWidth="1"/>
-    <col min="13" max="13" width="13.33203125" customWidth="1"/>
-    <col min="14" max="14" width="14.33203125" customWidth="1"/>
+    <col min="4" max="4" width="13.7109375" customWidth="1"/>
+    <col min="5" max="5" width="17.140625" customWidth="1"/>
+    <col min="6" max="6" width="16.140625" customWidth="1"/>
+    <col min="7" max="7" width="85.42578125" customWidth="1"/>
+    <col min="8" max="8" width="25.42578125" customWidth="1"/>
+    <col min="11" max="11" width="13.28515625" customWidth="1"/>
+    <col min="12" max="12" width="43.85546875" customWidth="1"/>
+    <col min="13" max="13" width="13.28515625" customWidth="1"/>
+    <col min="14" max="14" width="14.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="15.6">
+    <row r="1" spans="1:9" ht="15.75">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1143,7 +1146,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="15.6">
+    <row r="3" spans="1:9" ht="15.75">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
@@ -1205,7 +1208,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="15.6">
+    <row r="10" spans="1:9" ht="15.75">
       <c r="A10" s="1" t="s">
         <v>10</v>
       </c>
@@ -1261,7 +1264,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="13" spans="1:9" ht="15.6">
+    <row r="13" spans="1:9" ht="15.75">
       <c r="A13" s="3" t="s">
         <v>74</v>
       </c>
@@ -1308,7 +1311,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="15" spans="1:9" ht="15.6">
+    <row r="15" spans="1:9" ht="15.75">
       <c r="A15" s="3" t="s">
         <v>64</v>
       </c>
@@ -1353,7 +1356,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="18" spans="1:9" ht="15.6">
+    <row r="18" spans="1:9" ht="15.75">
       <c r="A18" s="1" t="s">
         <v>2</v>
       </c>
@@ -1415,7 +1418,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="25" spans="1:9" ht="15.6">
+    <row r="25" spans="1:9" ht="15.75">
       <c r="A25" s="1" t="s">
         <v>10</v>
       </c>
@@ -1471,7 +1474,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="28" spans="1:9" ht="15.6">
+    <row r="28" spans="1:9" ht="15.75">
       <c r="A28" s="3" t="s">
         <v>74</v>
       </c>
@@ -1518,7 +1521,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="30" spans="1:9" ht="15.6">
+    <row r="30" spans="1:9" ht="15.75">
       <c r="A30" s="3" t="s">
         <v>64</v>
       </c>
@@ -1563,7 +1566,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="33" spans="1:8" ht="15.6">
+    <row r="33" spans="1:8" ht="15.75">
       <c r="A33" s="4" t="s">
         <v>2</v>
       </c>
@@ -1689,7 +1692,7 @@
       <c r="G41" s="5"/>
       <c r="H41" s="5"/>
     </row>
-    <row r="42" spans="1:8" ht="15.6">
+    <row r="42" spans="1:8" ht="15.75">
       <c r="A42" s="4" t="s">
         <v>10</v>
       </c>
@@ -2152,7 +2155,7 @@
       </c>
       <c r="H61" s="5"/>
     </row>
-    <row r="63" spans="1:8" ht="15.6">
+    <row r="63" spans="1:8" ht="15.75">
       <c r="A63" s="4" t="s">
         <v>2</v>
       </c>
@@ -2278,7 +2281,7 @@
       <c r="G71" s="5"/>
       <c r="H71" s="5"/>
     </row>
-    <row r="72" spans="1:8" ht="15.6">
+    <row r="72" spans="1:8" ht="15.75">
       <c r="A72" s="4" t="s">
         <v>10</v>
       </c>
@@ -2901,7 +2904,7 @@
       <c r="K100" s="15"/>
       <c r="L100" s="15"/>
     </row>
-    <row r="101" spans="1:12" ht="15.6">
+    <row r="101" spans="1:12" ht="15.75">
       <c r="A101" s="3" t="s">
         <v>64</v>
       </c>
@@ -3597,7 +3600,9 @@
       <c r="G132" s="15" t="s">
         <v>157</v>
       </c>
-      <c r="H132" s="15"/>
+      <c r="H132" s="15" t="s">
+        <v>216</v>
+      </c>
       <c r="I132" s="15"/>
       <c r="J132" s="15"/>
       <c r="K132" s="15"/>
@@ -3631,53 +3636,62 @@
       <c r="K133" s="15"/>
       <c r="L133" s="15"/>
     </row>
-    <row r="134" spans="1:12">
-      <c r="A134" s="15" t="s">
-        <v>69</v>
-      </c>
-      <c r="B134" s="16">
+    <row r="134" spans="1:12" ht="15.75">
+      <c r="A134" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="B134">
+        <f>B135</f>
         <v>5.0000000000000001E-3</v>
       </c>
-      <c r="C134" s="15"/>
-      <c r="D134" s="15" t="s">
-        <v>21</v>
-      </c>
-      <c r="E134" s="12" t="s">
-        <v>30</v>
-      </c>
-      <c r="F134" s="15" t="s">
-        <v>22</v>
-      </c>
-      <c r="G134" s="15"/>
-      <c r="H134" s="15" t="s">
-        <v>196</v>
-      </c>
-      <c r="I134" s="15"/>
+      <c r="C134" t="s">
+        <v>67</v>
+      </c>
+      <c r="D134" t="s">
+        <v>21</v>
+      </c>
+      <c r="F134" t="s">
+        <v>17</v>
+      </c>
+      <c r="G134" t="s">
+        <v>65</v>
+      </c>
+      <c r="H134" t="s">
+        <v>72</v>
+      </c>
       <c r="J134" s="15"/>
       <c r="K134" s="15"/>
       <c r="L134" s="15"/>
     </row>
     <row r="135" spans="1:12">
-      <c r="A135" s="15"/>
-      <c r="B135" s="12"/>
+      <c r="A135" s="15" t="s">
+        <v>69</v>
+      </c>
+      <c r="B135" s="16">
+        <v>5.0000000000000001E-3</v>
+      </c>
       <c r="C135" s="15"/>
-      <c r="D135" s="15"/>
-      <c r="E135" s="15"/>
-      <c r="F135" s="15"/>
+      <c r="D135" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="E135" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="F135" s="15" t="s">
+        <v>22</v>
+      </c>
       <c r="G135" s="15"/>
-      <c r="H135" s="15"/>
+      <c r="H135" s="15" t="s">
+        <v>196</v>
+      </c>
       <c r="I135" s="15"/>
       <c r="J135" s="15"/>
       <c r="K135" s="15"/>
       <c r="L135" s="15"/>
     </row>
     <row r="136" spans="1:12">
-      <c r="A136" s="15" t="s">
-        <v>2</v>
-      </c>
-      <c r="B136" s="13" t="s">
-        <v>145</v>
-      </c>
+      <c r="A136" s="15"/>
+      <c r="B136" s="12"/>
       <c r="C136" s="15"/>
       <c r="D136" s="15"/>
       <c r="E136" s="15"/>
@@ -3691,10 +3705,10 @@
     </row>
     <row r="137" spans="1:12">
       <c r="A137" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="B137" s="15" t="s">
-        <v>182</v>
+        <v>2</v>
+      </c>
+      <c r="B137" s="13" t="s">
+        <v>145</v>
       </c>
       <c r="C137" s="15"/>
       <c r="D137" s="15"/>
@@ -3709,10 +3723,10 @@
     </row>
     <row r="138" spans="1:12">
       <c r="A138" s="15" t="s">
-        <v>51</v>
+        <v>6</v>
       </c>
       <c r="B138" s="15" t="s">
-        <v>205</v>
+        <v>182</v>
       </c>
       <c r="C138" s="15"/>
       <c r="D138" s="15"/>
@@ -3726,11 +3740,11 @@
       <c r="L138" s="15"/>
     </row>
     <row r="139" spans="1:12">
-      <c r="A139" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="B139" s="5" t="s">
-        <v>53</v>
+      <c r="A139" s="15" t="s">
+        <v>51</v>
+      </c>
+      <c r="B139" s="15" t="s">
+        <v>205</v>
       </c>
       <c r="C139" s="15"/>
       <c r="D139" s="15"/>
@@ -3744,11 +3758,11 @@
       <c r="L139" s="15"/>
     </row>
     <row r="140" spans="1:12">
-      <c r="A140" s="15" t="s">
-        <v>7</v>
-      </c>
-      <c r="B140" s="15" t="s">
-        <v>8</v>
+      <c r="A140" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="B140" s="5" t="s">
+        <v>53</v>
       </c>
       <c r="C140" s="15"/>
       <c r="D140" s="15"/>
@@ -3763,10 +3777,10 @@
     </row>
     <row r="141" spans="1:12">
       <c r="A141" s="15" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="B141" s="15" t="s">
-        <v>145</v>
+        <v>8</v>
       </c>
       <c r="C141" s="15"/>
       <c r="D141" s="15"/>
@@ -3781,10 +3795,10 @@
     </row>
     <row r="142" spans="1:12">
       <c r="A142" s="15" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B142" s="15" t="s">
-        <v>13</v>
+        <v>145</v>
       </c>
       <c r="C142" s="15"/>
       <c r="D142" s="15"/>
@@ -3799,9 +3813,11 @@
     </row>
     <row r="143" spans="1:12">
       <c r="A143" s="15" t="s">
-        <v>10</v>
-      </c>
-      <c r="B143" s="15"/>
+        <v>13</v>
+      </c>
+      <c r="B143" s="15" t="s">
+        <v>13</v>
+      </c>
       <c r="C143" s="15"/>
       <c r="D143" s="15"/>
       <c r="E143" s="15"/>
@@ -3815,32 +3831,16 @@
     </row>
     <row r="144" spans="1:12">
       <c r="A144" s="15" t="s">
-        <v>11</v>
-      </c>
-      <c r="B144" s="15" t="s">
-        <v>12</v>
-      </c>
-      <c r="C144" s="15" t="s">
-        <v>7</v>
-      </c>
-      <c r="D144" s="15" t="s">
-        <v>13</v>
-      </c>
-      <c r="E144" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="F144" s="15" t="s">
-        <v>9</v>
-      </c>
-      <c r="G144" s="15" t="s">
-        <v>14</v>
-      </c>
-      <c r="H144" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="I144" s="15" t="s">
-        <v>18</v>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="B144" s="15"/>
+      <c r="C144" s="15"/>
+      <c r="D144" s="15"/>
+      <c r="E144" s="15"/>
+      <c r="F144" s="15"/>
+      <c r="G144" s="15"/>
+      <c r="H144" s="15"/>
+      <c r="I144" s="15"/>
       <c r="J144" s="15" t="s">
         <v>133</v>
       </c>
@@ -3852,109 +3852,113 @@
       </c>
     </row>
     <row r="145" spans="1:12">
-      <c r="A145" s="15" t="str">
-        <f>B141</f>
-        <v>gaseous hydrogen production</v>
-      </c>
-      <c r="B145" s="16">
-        <v>1</v>
+      <c r="A145" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="B145" s="15" t="s">
+        <v>12</v>
       </c>
       <c r="C145" s="15" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D145" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="E145" s="15"/>
+      <c r="E145" s="15" t="s">
+        <v>19</v>
+      </c>
       <c r="F145" s="15" t="s">
-        <v>16</v>
-      </c>
-      <c r="G145" s="15" t="str">
-        <f>B141</f>
-        <v>gaseous hydrogen production</v>
+        <v>9</v>
+      </c>
+      <c r="G145" s="15" t="s">
+        <v>14</v>
       </c>
       <c r="H145" s="15" t="s">
-        <v>136</v>
-      </c>
-      <c r="I145" s="15"/>
+        <v>6</v>
+      </c>
+      <c r="I145" s="15" t="s">
+        <v>18</v>
+      </c>
       <c r="J145" s="15"/>
       <c r="K145" s="15"/>
       <c r="L145" s="15"/>
     </row>
     <row r="146" spans="1:12">
-      <c r="A146" s="15" t="s">
-        <v>64</v>
-      </c>
-      <c r="B146">
-        <f>B149</f>
-        <v>3.0000000000000001E-3</v>
-      </c>
-      <c r="C146" t="s">
-        <v>67</v>
-      </c>
-      <c r="D146" t="s">
-        <v>21</v>
-      </c>
-      <c r="F146" t="s">
-        <v>17</v>
-      </c>
-      <c r="G146" t="s">
-        <v>65</v>
-      </c>
-      <c r="H146" t="s">
-        <v>72</v>
-      </c>
+      <c r="A146" s="15" t="str">
+        <f>B142</f>
+        <v>gaseous hydrogen production</v>
+      </c>
+      <c r="B146" s="16">
+        <v>1</v>
+      </c>
+      <c r="C146" s="15" t="s">
+        <v>8</v>
+      </c>
+      <c r="D146" s="15" t="s">
+        <v>13</v>
+      </c>
+      <c r="E146" s="15"/>
+      <c r="F146" s="15" t="s">
+        <v>16</v>
+      </c>
+      <c r="G146" s="15" t="str">
+        <f>B142</f>
+        <v>gaseous hydrogen production</v>
+      </c>
+      <c r="H146" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="I146" s="15"/>
     </row>
     <row r="147" spans="1:12">
       <c r="A147" s="15" t="s">
-        <v>198</v>
-      </c>
-      <c r="B147" s="17">
-        <v>3.4299999999999999E-9</v>
-      </c>
-      <c r="C147" s="15" t="s">
+        <v>64</v>
+      </c>
+      <c r="B147">
+        <f>B150</f>
+        <v>3.0000000000000001E-3</v>
+      </c>
+      <c r="C147" t="s">
         <v>67</v>
       </c>
-      <c r="D147" s="15" t="s">
-        <v>13</v>
-      </c>
-      <c r="E147" s="15"/>
-      <c r="F147" s="15" t="s">
+      <c r="D147" t="s">
+        <v>21</v>
+      </c>
+      <c r="F147" t="s">
         <v>17</v>
       </c>
       <c r="G147" t="s">
-        <v>199</v>
-      </c>
-      <c r="H147" s="15" t="s">
-        <v>201</v>
-      </c>
-      <c r="I147" s="15"/>
+        <v>65</v>
+      </c>
+      <c r="H147" t="s">
+        <v>72</v>
+      </c>
       <c r="J147" s="15"/>
       <c r="K147" s="15"/>
       <c r="L147" s="15"/>
     </row>
     <row r="148" spans="1:12">
       <c r="A148" s="15" t="s">
-        <v>139</v>
-      </c>
-      <c r="B148" s="16">
-        <v>1.25</v>
+        <v>198</v>
+      </c>
+      <c r="B148" s="17">
+        <v>3.4299999999999999E-9</v>
       </c>
       <c r="C148" s="15" t="s">
-        <v>8</v>
+        <v>67</v>
       </c>
       <c r="D148" s="15" t="s">
-        <v>66</v>
+        <v>13</v>
       </c>
       <c r="E148" s="15"/>
       <c r="F148" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="G148" s="15" t="s">
-        <v>157</v>
+      <c r="G148" t="s">
+        <v>199</v>
       </c>
       <c r="H148" s="15" t="s">
-        <v>146</v>
+        <v>201</v>
       </c>
       <c r="I148" s="15"/>
       <c r="J148" s="15"/>
@@ -3963,22 +3967,24 @@
     </row>
     <row r="149" spans="1:12">
       <c r="A149" s="15" t="s">
-        <v>69</v>
+        <v>139</v>
       </c>
       <c r="B149" s="16">
-        <v>3.0000000000000001E-3</v>
-      </c>
-      <c r="C149" s="15"/>
+        <v>1.25</v>
+      </c>
+      <c r="C149" s="15" t="s">
+        <v>8</v>
+      </c>
       <c r="D149" s="15" t="s">
-        <v>21</v>
-      </c>
-      <c r="E149" s="12" t="s">
-        <v>30</v>
-      </c>
+        <v>66</v>
+      </c>
+      <c r="E149" s="15"/>
       <c r="F149" s="15" t="s">
-        <v>22</v>
-      </c>
-      <c r="G149" s="15"/>
+        <v>17</v>
+      </c>
+      <c r="G149" s="15" t="s">
+        <v>157</v>
+      </c>
       <c r="H149" s="15" t="s">
         <v>146</v>
       </c>
@@ -3989,17 +3995,17 @@
     </row>
     <row r="150" spans="1:12">
       <c r="A150" s="15" t="s">
-        <v>152</v>
-      </c>
-      <c r="B150" s="12">
-        <v>3.8000000000000002E-4</v>
+        <v>69</v>
+      </c>
+      <c r="B150" s="16">
+        <v>3.0000000000000001E-3</v>
       </c>
       <c r="C150" s="15"/>
       <c r="D150" s="15" t="s">
-        <v>142</v>
-      </c>
-      <c r="E150" s="15" t="s">
-        <v>147</v>
+        <v>21</v>
+      </c>
+      <c r="E150" s="12" t="s">
+        <v>30</v>
       </c>
       <c r="F150" s="15" t="s">
         <v>22</v>
@@ -4015,17 +4021,17 @@
     </row>
     <row r="151" spans="1:12">
       <c r="A151" s="15" t="s">
-        <v>149</v>
-      </c>
-      <c r="B151" s="15">
-        <v>9.4600000000000004E-2</v>
+        <v>152</v>
+      </c>
+      <c r="B151" s="12">
+        <v>3.8000000000000002E-4</v>
       </c>
       <c r="C151" s="15"/>
       <c r="D151" s="15" t="s">
         <v>142</v>
       </c>
       <c r="E151" s="15" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="F151" s="15" t="s">
         <v>22</v>
@@ -4041,17 +4047,17 @@
     </row>
     <row r="152" spans="1:12">
       <c r="A152" s="15" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B152" s="15">
-        <v>9.5000000000000001E-2</v>
+        <v>9.4600000000000004E-2</v>
       </c>
       <c r="C152" s="15"/>
       <c r="D152" s="15" t="s">
         <v>142</v>
       </c>
       <c r="E152" s="15" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="F152" s="15" t="s">
         <v>22</v>
@@ -4066,26 +4072,34 @@
       <c r="L152" s="15"/>
     </row>
     <row r="153" spans="1:12">
-      <c r="A153" s="15"/>
-      <c r="B153" s="15"/>
+      <c r="A153" s="15" t="s">
+        <v>150</v>
+      </c>
+      <c r="B153" s="15">
+        <v>9.5000000000000001E-2</v>
+      </c>
       <c r="C153" s="15"/>
-      <c r="D153" s="15"/>
-      <c r="E153" s="15"/>
-      <c r="F153" s="15"/>
+      <c r="D153" s="15" t="s">
+        <v>142</v>
+      </c>
+      <c r="E153" s="15" t="s">
+        <v>151</v>
+      </c>
+      <c r="F153" s="15" t="s">
+        <v>22</v>
+      </c>
       <c r="G153" s="15"/>
-      <c r="H153" s="15"/>
+      <c r="H153" s="15" t="s">
+        <v>146</v>
+      </c>
       <c r="I153" s="15"/>
       <c r="J153" s="15"/>
       <c r="K153" s="15"/>
       <c r="L153" s="15"/>
     </row>
     <row r="154" spans="1:12">
-      <c r="A154" s="15" t="s">
-        <v>2</v>
-      </c>
-      <c r="B154" s="13" t="s">
-        <v>160</v>
-      </c>
+      <c r="A154" s="15"/>
+      <c r="B154" s="15"/>
       <c r="C154" s="15"/>
       <c r="D154" s="15"/>
       <c r="E154" s="15"/>
@@ -4099,10 +4113,10 @@
     </row>
     <row r="155" spans="1:12">
       <c r="A155" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="B155" t="s">
-        <v>209</v>
+        <v>2</v>
+      </c>
+      <c r="B155" s="13" t="s">
+        <v>160</v>
       </c>
       <c r="C155" s="15"/>
       <c r="D155" s="15"/>
@@ -4117,10 +4131,10 @@
     </row>
     <row r="156" spans="1:12">
       <c r="A156" s="15" t="s">
-        <v>51</v>
-      </c>
-      <c r="B156" s="15" t="s">
-        <v>167</v>
+        <v>6</v>
+      </c>
+      <c r="B156" t="s">
+        <v>209</v>
       </c>
       <c r="C156" s="15"/>
       <c r="D156" s="15"/>
@@ -4134,11 +4148,11 @@
       <c r="L156" s="15"/>
     </row>
     <row r="157" spans="1:12">
-      <c r="A157" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="B157" s="5" t="s">
-        <v>53</v>
+      <c r="A157" s="15" t="s">
+        <v>51</v>
+      </c>
+      <c r="B157" s="15" t="s">
+        <v>167</v>
       </c>
       <c r="C157" s="15"/>
       <c r="D157" s="15"/>
@@ -4152,11 +4166,11 @@
       <c r="L157" s="15"/>
     </row>
     <row r="158" spans="1:12">
-      <c r="A158" s="15" t="s">
-        <v>7</v>
-      </c>
-      <c r="B158" s="15" t="s">
-        <v>8</v>
+      <c r="A158" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="B158" s="5" t="s">
+        <v>53</v>
       </c>
       <c r="C158" s="15"/>
       <c r="D158" s="15"/>
@@ -4171,10 +4185,10 @@
     </row>
     <row r="159" spans="1:12">
       <c r="A159" s="15" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="B159" s="15" t="s">
-        <v>160</v>
+        <v>8</v>
       </c>
       <c r="C159" s="15"/>
       <c r="D159" s="15"/>
@@ -4189,10 +4203,10 @@
     </row>
     <row r="160" spans="1:12">
       <c r="A160" s="15" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B160" s="15" t="s">
-        <v>13</v>
+        <v>160</v>
       </c>
       <c r="C160" s="15"/>
       <c r="D160" s="15"/>
@@ -4207,9 +4221,11 @@
     </row>
     <row r="161" spans="1:12">
       <c r="A161" s="15" t="s">
-        <v>10</v>
-      </c>
-      <c r="B161" s="15"/>
+        <v>13</v>
+      </c>
+      <c r="B161" s="15" t="s">
+        <v>13</v>
+      </c>
       <c r="C161" s="15"/>
       <c r="D161" s="15"/>
       <c r="E161" s="15"/>
@@ -4223,32 +4239,16 @@
     </row>
     <row r="162" spans="1:12">
       <c r="A162" s="15" t="s">
-        <v>11</v>
-      </c>
-      <c r="B162" s="15" t="s">
-        <v>12</v>
-      </c>
-      <c r="C162" s="15" t="s">
-        <v>7</v>
-      </c>
-      <c r="D162" s="15" t="s">
-        <v>13</v>
-      </c>
-      <c r="E162" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="F162" s="15" t="s">
-        <v>9</v>
-      </c>
-      <c r="G162" s="15" t="s">
-        <v>14</v>
-      </c>
-      <c r="H162" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="I162" s="15" t="s">
-        <v>18</v>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="B162" s="15"/>
+      <c r="C162" s="15"/>
+      <c r="D162" s="15"/>
+      <c r="E162" s="15"/>
+      <c r="F162" s="15"/>
+      <c r="G162" s="15"/>
+      <c r="H162" s="15"/>
+      <c r="I162" s="15"/>
       <c r="J162" s="15" t="s">
         <v>133</v>
       </c>
@@ -4260,42 +4260,44 @@
       </c>
     </row>
     <row r="163" spans="1:12">
-      <c r="A163" s="15" t="str">
-        <f>B159</f>
-        <v>ammonia cracking</v>
-      </c>
-      <c r="B163" s="16">
-        <v>1</v>
+      <c r="A163" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="B163" s="15" t="s">
+        <v>12</v>
       </c>
       <c r="C163" s="15" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D163" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="E163" s="15"/>
+      <c r="E163" s="15" t="s">
+        <v>19</v>
+      </c>
       <c r="F163" s="15" t="s">
-        <v>16</v>
-      </c>
-      <c r="G163" s="15" t="str">
-        <f>B159</f>
-        <v>ammonia cracking</v>
+        <v>9</v>
+      </c>
+      <c r="G163" s="15" t="s">
+        <v>14</v>
       </c>
       <c r="H163" s="15" t="s">
-        <v>136</v>
-      </c>
-      <c r="I163" s="15"/>
+        <v>6</v>
+      </c>
+      <c r="I163" s="15" t="s">
+        <v>18</v>
+      </c>
       <c r="J163" s="15"/>
       <c r="K163" s="15"/>
       <c r="L163" s="15"/>
     </row>
     <row r="164" spans="1:12">
-      <c r="A164" s="15" t="s">
-        <v>161</v>
-      </c>
-      <c r="B164" s="17">
-        <f>1/(28*1000*300*50)</f>
-        <v>2.380952380952381E-9</v>
+      <c r="A164" s="15" t="str">
+        <f>B160</f>
+        <v>ammonia cracking</v>
+      </c>
+      <c r="B164" s="16">
+        <v>1</v>
       </c>
       <c r="C164" s="15" t="s">
         <v>8</v>
@@ -4305,13 +4307,14 @@
       </c>
       <c r="E164" s="15"/>
       <c r="F164" s="15" t="s">
-        <v>17</v>
-      </c>
-      <c r="G164" s="15" t="s">
-        <v>162</v>
+        <v>16</v>
+      </c>
+      <c r="G164" s="15" t="str">
+        <f>B160</f>
+        <v>ammonia cracking</v>
       </c>
       <c r="H164" s="15" t="s">
-        <v>166</v>
+        <v>136</v>
       </c>
       <c r="I164" s="15"/>
       <c r="J164" s="15"/>
@@ -4320,7 +4323,7 @@
     </row>
     <row r="165" spans="1:12">
       <c r="A165" s="15" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="B165" s="17">
         <f>1/(28*1000*300*50)</f>
@@ -4337,10 +4340,10 @@
         <v>17</v>
       </c>
       <c r="G165" s="15" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="H165" s="15" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="I165" s="15"/>
       <c r="J165" s="15"/>
@@ -4348,118 +4351,115 @@
       <c r="L165" s="15"/>
     </row>
     <row r="166" spans="1:12">
-      <c r="A166" t="s">
+      <c r="A166" s="15" t="s">
+        <v>163</v>
+      </c>
+      <c r="B166" s="17">
+        <f>1/(28*1000*300*50)</f>
+        <v>2.380952380952381E-9</v>
+      </c>
+      <c r="C166" s="15" t="s">
+        <v>8</v>
+      </c>
+      <c r="D166" s="15" t="s">
+        <v>13</v>
+      </c>
+      <c r="E166" s="15"/>
+      <c r="F166" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="G166" s="15" t="s">
+        <v>164</v>
+      </c>
+      <c r="H166" s="15" t="s">
+        <v>165</v>
+      </c>
+      <c r="I166" s="15"/>
+    </row>
+    <row r="167" spans="1:12">
+      <c r="A167" t="s">
         <v>76</v>
       </c>
-      <c r="B166" s="18">
-        <f>3.086+0.6</f>
-        <v>3.6859999999999999</v>
-      </c>
-      <c r="C166" t="s">
+      <c r="B167" s="18">
+        <f>(3.086/7.67)+0.6</f>
+        <v>1.0023468057366363</v>
+      </c>
+      <c r="C167" t="s">
         <v>67</v>
       </c>
-      <c r="D166" t="s">
+      <c r="D167" t="s">
         <v>66</v>
       </c>
-      <c r="F166" t="s">
+      <c r="F167" t="s">
         <v>17</v>
       </c>
-      <c r="G166" t="s">
+      <c r="G167" t="s">
         <v>62</v>
       </c>
-      <c r="H166" t="s">
+      <c r="H167" t="s">
         <v>210</v>
-      </c>
-    </row>
-    <row r="168" spans="1:12">
-      <c r="A168" t="s">
-        <v>2</v>
-      </c>
-      <c r="B168" s="13" t="s">
-        <v>168</v>
       </c>
     </row>
     <row r="169" spans="1:12">
       <c r="A169" t="s">
-        <v>6</v>
-      </c>
-      <c r="B169" t="s">
-        <v>181</v>
+        <v>2</v>
+      </c>
+      <c r="B169" s="13" t="s">
+        <v>168</v>
       </c>
     </row>
     <row r="170" spans="1:12">
       <c r="A170" t="s">
+        <v>6</v>
+      </c>
+      <c r="B170" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="171" spans="1:12">
+      <c r="A171" t="s">
         <v>51</v>
       </c>
-      <c r="B170" t="s">
+      <c r="B171" t="s">
         <v>202</v>
       </c>
     </row>
-    <row r="171" spans="1:12">
-      <c r="A171" s="5" t="s">
+    <row r="172" spans="1:12">
+      <c r="A172" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="B171" s="12" t="s">
+      <c r="B172" s="12" t="s">
         <v>208</v>
-      </c>
-    </row>
-    <row r="172" spans="1:12">
-      <c r="A172" t="s">
-        <v>7</v>
-      </c>
-      <c r="B172" t="s">
-        <v>8</v>
       </c>
     </row>
     <row r="173" spans="1:12">
       <c r="A173" t="s">
-        <v>14</v>
-      </c>
-      <c r="B173" t="str">
-        <f>B168</f>
-        <v>liquid ammonia production</v>
+        <v>7</v>
+      </c>
+      <c r="B173" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="174" spans="1:12">
       <c r="A174" t="s">
-        <v>13</v>
-      </c>
-      <c r="B174" t="s">
-        <v>13</v>
+        <v>14</v>
+      </c>
+      <c r="B174" t="str">
+        <f>B169</f>
+        <v>liquid ammonia production</v>
       </c>
     </row>
     <row r="175" spans="1:12">
       <c r="A175" t="s">
-        <v>10</v>
+        <v>13</v>
+      </c>
+      <c r="B175" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="176" spans="1:12">
       <c r="A176" t="s">
-        <v>11</v>
-      </c>
-      <c r="B176" t="s">
-        <v>12</v>
-      </c>
-      <c r="C176" t="s">
-        <v>7</v>
-      </c>
-      <c r="D176" t="s">
-        <v>13</v>
-      </c>
-      <c r="E176" t="s">
-        <v>19</v>
-      </c>
-      <c r="F176" t="s">
-        <v>9</v>
-      </c>
-      <c r="G176" t="s">
-        <v>14</v>
-      </c>
-      <c r="H176" t="s">
-        <v>6</v>
-      </c>
-      <c r="I176" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="J176" t="s">
         <v>133</v>
@@ -4471,59 +4471,65 @@
         <v>135</v>
       </c>
     </row>
-    <row r="177" spans="1:8">
-      <c r="A177" t="str">
-        <f>B173</f>
-        <v>liquid ammonia production</v>
-      </c>
-      <c r="B177" s="18">
-        <v>1</v>
+    <row r="177" spans="1:9">
+      <c r="A177" t="s">
+        <v>11</v>
+      </c>
+      <c r="B177" t="s">
+        <v>12</v>
       </c>
       <c r="C177" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D177" t="s">
         <v>13</v>
       </c>
+      <c r="E177" t="s">
+        <v>19</v>
+      </c>
       <c r="F177" t="s">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="G177" t="s">
-        <v>169</v>
+        <v>14</v>
       </c>
       <c r="H177" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="178" spans="1:8">
-      <c r="A178" t="s">
-        <v>172</v>
+        <v>6</v>
+      </c>
+      <c r="I177" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="178" spans="1:9">
+      <c r="A178" t="str">
+        <f>B174</f>
+        <v>liquid ammonia production</v>
       </c>
       <c r="B178" s="18">
-        <v>0.81499999999999995</v>
+        <v>1</v>
       </c>
       <c r="C178" t="s">
         <v>8</v>
       </c>
       <c r="D178" t="s">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="F178" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G178" t="s">
+        <v>169</v>
+      </c>
+      <c r="H178" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="179" spans="1:9">
+      <c r="A179" t="s">
         <v>172</v>
       </c>
-      <c r="H178" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="179" spans="1:8">
-      <c r="A179" t="s">
-        <v>173</v>
-      </c>
       <c r="B179" s="18">
-        <v>5.1499999999999998E-5</v>
+        <v>0.81499999999999995</v>
       </c>
       <c r="C179" t="s">
         <v>8</v>
@@ -4535,112 +4541,118 @@
         <v>17</v>
       </c>
       <c r="G179" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="H179" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="180" spans="1:8">
+    <row r="180" spans="1:9">
       <c r="A180" t="s">
-        <v>163</v>
+        <v>173</v>
       </c>
       <c r="B180" s="18">
-        <v>3.29E-10</v>
+        <v>5.1499999999999998E-5</v>
       </c>
       <c r="C180" t="s">
         <v>8</v>
       </c>
       <c r="D180" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="F180" t="s">
         <v>17</v>
       </c>
       <c r="G180" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="181" spans="1:8">
+        <v>173</v>
+      </c>
+      <c r="H180" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="181" spans="1:9">
       <c r="A181" t="s">
-        <v>139</v>
+        <v>163</v>
       </c>
       <c r="B181" s="18">
-        <v>1.44</v>
+        <v>3.29E-10</v>
       </c>
       <c r="C181" t="s">
         <v>8</v>
       </c>
       <c r="D181" t="s">
-        <v>66</v>
+        <v>13</v>
       </c>
       <c r="F181" t="s">
         <v>17</v>
       </c>
       <c r="G181" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="182" spans="1:8">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="182" spans="1:9">
       <c r="A182" t="s">
-        <v>174</v>
+        <v>139</v>
       </c>
       <c r="B182" s="18">
-        <v>5.1499999999999998E-5</v>
+        <v>1.44</v>
       </c>
       <c r="C182" t="s">
-        <v>131</v>
+        <v>8</v>
       </c>
       <c r="D182" t="s">
-        <v>21</v>
+        <v>66</v>
       </c>
       <c r="F182" t="s">
         <v>17</v>
       </c>
       <c r="G182" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="183" spans="1:9">
+      <c r="A183" t="s">
+        <v>174</v>
+      </c>
+      <c r="B183" s="18">
+        <v>5.1499999999999998E-5</v>
+      </c>
+      <c r="C183" t="s">
+        <v>131</v>
+      </c>
+      <c r="D183" t="s">
+        <v>21</v>
+      </c>
+      <c r="F183" t="s">
+        <v>17</v>
+      </c>
+      <c r="G183" t="s">
         <v>190</v>
       </c>
     </row>
-    <row r="183" spans="1:8">
-      <c r="A183" t="s">
+    <row r="184" spans="1:9">
+      <c r="A184" t="s">
         <v>150</v>
       </c>
-      <c r="B183" s="18">
+      <c r="B184" s="18">
         <v>0.14899999999999999</v>
       </c>
-      <c r="D183" t="s">
+      <c r="D184" t="s">
         <v>142</v>
       </c>
-      <c r="E183" s="15" t="s">
+      <c r="E184" s="15" t="s">
         <v>151</v>
-      </c>
-      <c r="F183" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="184" spans="1:8">
-      <c r="A184" t="s">
-        <v>69</v>
-      </c>
-      <c r="B184" s="18">
-        <v>7.67E-4</v>
-      </c>
-      <c r="D184" t="s">
-        <v>21</v>
-      </c>
-      <c r="E184" s="12" t="s">
-        <v>30</v>
       </c>
       <c r="F184" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="185" spans="1:8">
+    <row r="185" spans="1:9">
       <c r="A185" t="s">
-        <v>20</v>
+        <v>69</v>
       </c>
       <c r="B185" s="18">
-        <v>1.6299999999999999E-3</v>
+        <v>7.67E-4</v>
       </c>
       <c r="D185" t="s">
         <v>21</v>
@@ -4652,12 +4664,12 @@
         <v>22</v>
       </c>
     </row>
-    <row r="186" spans="1:8">
+    <row r="186" spans="1:9">
       <c r="A186" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="B186" s="18">
-        <v>1E-3</v>
+        <v>1.6299999999999999E-3</v>
       </c>
       <c r="D186" t="s">
         <v>21</v>
@@ -4669,15 +4681,15 @@
         <v>22</v>
       </c>
     </row>
-    <row r="187" spans="1:8">
+    <row r="187" spans="1:9">
       <c r="A187" t="s">
-        <v>149</v>
+        <v>25</v>
       </c>
       <c r="B187" s="18">
-        <v>4.7600000000000003E-2</v>
+        <v>1E-3</v>
       </c>
       <c r="D187" t="s">
-        <v>142</v>
+        <v>21</v>
       </c>
       <c r="E187" s="12" t="s">
         <v>30</v>
@@ -4686,111 +4698,99 @@
         <v>22</v>
       </c>
     </row>
-    <row r="188" spans="1:8">
+    <row r="188" spans="1:9">
       <c r="A188" t="s">
         <v>149</v>
       </c>
       <c r="B188" s="18">
-        <v>0.10100000000000001</v>
+        <v>4.7600000000000003E-2</v>
       </c>
       <c r="D188" t="s">
         <v>142</v>
       </c>
-      <c r="E188" s="15" t="s">
-        <v>148</v>
+      <c r="E188" s="12" t="s">
+        <v>30</v>
       </c>
       <c r="F188" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="190" spans="1:8">
-      <c r="A190" t="s">
+    <row r="189" spans="1:9">
+      <c r="A189" t="s">
+        <v>149</v>
+      </c>
+      <c r="B189" s="18">
+        <v>0.10100000000000001</v>
+      </c>
+      <c r="D189" t="s">
+        <v>142</v>
+      </c>
+      <c r="E189" s="15" t="s">
+        <v>148</v>
+      </c>
+      <c r="F189" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="191" spans="1:9">
+      <c r="A191" t="s">
         <v>2</v>
       </c>
-      <c r="B190" s="13" t="s">
+      <c r="B191" s="13" t="s">
         <v>172</v>
       </c>
     </row>
-    <row r="191" spans="1:8">
-      <c r="A191" t="s">
+    <row r="192" spans="1:9">
+      <c r="A192" t="s">
         <v>6</v>
       </c>
-      <c r="B191" t="s">
+      <c r="B192" t="s">
         <v>185</v>
       </c>
     </row>
-    <row r="192" spans="1:8">
-      <c r="A192" t="s">
+    <row r="193" spans="1:12">
+      <c r="A193" t="s">
         <v>51</v>
       </c>
-      <c r="B192" t="s">
+      <c r="B193" t="s">
         <v>203</v>
       </c>
     </row>
-    <row r="193" spans="1:12">
-      <c r="A193" s="5" t="s">
+    <row r="194" spans="1:12">
+      <c r="A194" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="B193" s="12" t="s">
+      <c r="B194" s="12" t="s">
         <v>207</v>
-      </c>
-    </row>
-    <row r="194" spans="1:12">
-      <c r="A194" t="s">
-        <v>7</v>
-      </c>
-      <c r="B194" t="s">
-        <v>8</v>
       </c>
     </row>
     <row r="195" spans="1:12">
       <c r="A195" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="B195" t="s">
-        <v>172</v>
+        <v>8</v>
       </c>
     </row>
     <row r="196" spans="1:12">
       <c r="A196" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B196" t="s">
-        <v>21</v>
+        <v>172</v>
       </c>
     </row>
     <row r="197" spans="1:12">
       <c r="A197" t="s">
-        <v>10</v>
+        <v>13</v>
+      </c>
+      <c r="B197" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="198" spans="1:12">
       <c r="A198" t="s">
-        <v>11</v>
-      </c>
-      <c r="B198" t="s">
-        <v>12</v>
-      </c>
-      <c r="C198" t="s">
-        <v>7</v>
-      </c>
-      <c r="D198" t="s">
-        <v>13</v>
-      </c>
-      <c r="E198" t="s">
-        <v>19</v>
-      </c>
-      <c r="F198" t="s">
-        <v>9</v>
-      </c>
-      <c r="G198" t="s">
-        <v>14</v>
-      </c>
-      <c r="H198" t="s">
-        <v>6</v>
-      </c>
-      <c r="I198" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="J198" t="s">
         <v>133</v>
@@ -4804,169 +4804,169 @@
     </row>
     <row r="199" spans="1:12">
       <c r="A199" t="s">
-        <v>172</v>
-      </c>
-      <c r="B199" s="18">
-        <v>1</v>
+        <v>11</v>
+      </c>
+      <c r="B199" t="s">
+        <v>12</v>
       </c>
       <c r="C199" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D199" t="s">
-        <v>21</v>
+        <v>13</v>
+      </c>
+      <c r="E199" t="s">
+        <v>19</v>
       </c>
       <c r="F199" t="s">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="G199" t="s">
-        <v>172</v>
+        <v>14</v>
       </c>
       <c r="H199" t="s">
-        <v>175</v>
+        <v>6</v>
+      </c>
+      <c r="I199" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="200" spans="1:12">
       <c r="A200" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="B200" s="18">
-        <v>4.4300000000000002E-10</v>
+        <v>1</v>
       </c>
       <c r="C200" t="s">
         <v>8</v>
       </c>
       <c r="D200" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="F200" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G200" t="s">
-        <v>188</v>
+        <v>172</v>
+      </c>
+      <c r="H200" t="s">
+        <v>175</v>
       </c>
     </row>
     <row r="201" spans="1:12">
       <c r="A201" t="s">
-        <v>150</v>
+        <v>176</v>
       </c>
       <c r="B201" s="18">
-        <v>4.0000000000000001E-3</v>
+        <v>4.4300000000000002E-10</v>
+      </c>
+      <c r="C201" t="s">
+        <v>8</v>
       </c>
       <c r="D201" t="s">
-        <v>142</v>
-      </c>
-      <c r="E201" s="15" t="s">
-        <v>151</v>
+        <v>13</v>
       </c>
       <c r="F201" t="s">
-        <v>22</v>
+        <v>17</v>
+      </c>
+      <c r="G201" t="s">
+        <v>188</v>
       </c>
     </row>
     <row r="202" spans="1:12">
       <c r="A202" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B202" s="18">
-        <v>2.4499999999999999E-3</v>
+        <v>4.0000000000000001E-3</v>
       </c>
       <c r="D202" t="s">
         <v>142</v>
       </c>
       <c r="E202" s="15" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="F202" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="204" spans="1:12">
-      <c r="A204" t="s">
-        <v>2</v>
-      </c>
-      <c r="B204" s="13" t="s">
-        <v>173</v>
+    <row r="203" spans="1:12">
+      <c r="A203" t="s">
+        <v>149</v>
+      </c>
+      <c r="B203" s="18">
+        <v>2.4499999999999999E-3</v>
+      </c>
+      <c r="D203" t="s">
+        <v>142</v>
+      </c>
+      <c r="E203" s="15" t="s">
+        <v>148</v>
+      </c>
+      <c r="F203" t="s">
+        <v>22</v>
       </c>
     </row>
     <row r="205" spans="1:12">
       <c r="A205" t="s">
-        <v>6</v>
-      </c>
-      <c r="B205" t="s">
-        <v>177</v>
+        <v>2</v>
+      </c>
+      <c r="B205" s="13" t="s">
+        <v>173</v>
       </c>
     </row>
     <row r="206" spans="1:12">
       <c r="A206" t="s">
+        <v>6</v>
+      </c>
+      <c r="B206" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="207" spans="1:12">
+      <c r="A207" t="s">
         <v>51</v>
       </c>
-      <c r="B206" t="s">
+      <c r="B207" t="s">
         <v>204</v>
       </c>
     </row>
-    <row r="207" spans="1:12">
-      <c r="A207" s="5" t="s">
+    <row r="208" spans="1:12">
+      <c r="A208" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="B207" s="12" t="s">
+      <c r="B208" s="12" t="s">
         <v>207</v>
-      </c>
-    </row>
-    <row r="208" spans="1:12">
-      <c r="A208" t="s">
-        <v>7</v>
-      </c>
-      <c r="B208" t="s">
-        <v>8</v>
       </c>
     </row>
     <row r="209" spans="1:12">
       <c r="A209" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="B209" t="s">
-        <v>173</v>
+        <v>8</v>
       </c>
     </row>
     <row r="210" spans="1:12">
       <c r="A210" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B210" t="s">
-        <v>21</v>
+        <v>173</v>
       </c>
     </row>
     <row r="211" spans="1:12">
       <c r="A211" t="s">
-        <v>10</v>
+        <v>13</v>
+      </c>
+      <c r="B211" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="212" spans="1:12">
       <c r="A212" t="s">
-        <v>11</v>
-      </c>
-      <c r="B212" t="s">
-        <v>12</v>
-      </c>
-      <c r="C212" t="s">
-        <v>7</v>
-      </c>
-      <c r="D212" t="s">
-        <v>13</v>
-      </c>
-      <c r="E212" t="s">
-        <v>19</v>
-      </c>
-      <c r="F212" t="s">
-        <v>9</v>
-      </c>
-      <c r="G212" t="s">
-        <v>14</v>
-      </c>
-      <c r="H212" t="s">
-        <v>6</v>
-      </c>
-      <c r="I212" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="J212" t="s">
         <v>133</v>
@@ -4980,33 +4980,39 @@
     </row>
     <row r="213" spans="1:12">
       <c r="A213" t="s">
-        <v>173</v>
-      </c>
-      <c r="B213" s="18">
-        <v>1</v>
+        <v>11</v>
+      </c>
+      <c r="B213" t="s">
+        <v>12</v>
       </c>
       <c r="C213" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D213" t="s">
-        <v>21</v>
+        <v>13</v>
+      </c>
+      <c r="E213" t="s">
+        <v>19</v>
       </c>
       <c r="F213" t="s">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="G213" t="s">
-        <v>173</v>
+        <v>14</v>
       </c>
       <c r="H213" t="s">
-        <v>178</v>
+        <v>6</v>
+      </c>
+      <c r="I213" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="214" spans="1:12">
       <c r="A214" t="s">
-        <v>179</v>
+        <v>173</v>
       </c>
       <c r="B214" s="18">
-        <v>0.91700000000000004</v>
+        <v>1</v>
       </c>
       <c r="C214" t="s">
         <v>8</v>
@@ -5015,21 +5021,24 @@
         <v>21</v>
       </c>
       <c r="F214" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G214" t="s">
-        <v>186</v>
+        <v>173</v>
+      </c>
+      <c r="H214" t="s">
+        <v>178</v>
       </c>
     </row>
     <row r="215" spans="1:12">
       <c r="A215" t="s">
-        <v>193</v>
+        <v>179</v>
       </c>
       <c r="B215" s="18">
-        <v>0.03</v>
+        <v>0.91700000000000004</v>
       </c>
       <c r="C215" t="s">
-        <v>67</v>
+        <v>8</v>
       </c>
       <c r="D215" t="s">
         <v>21</v>
@@ -5038,21 +5047,18 @@
         <v>17</v>
       </c>
       <c r="G215" t="s">
-        <v>191</v>
-      </c>
-      <c r="H215" t="s">
-        <v>192</v>
+        <v>186</v>
       </c>
     </row>
     <row r="216" spans="1:12">
       <c r="A216" t="s">
-        <v>180</v>
+        <v>193</v>
       </c>
       <c r="B216" s="18">
-        <v>5.2499999999999998E-2</v>
+        <v>0.03</v>
       </c>
       <c r="C216" t="s">
-        <v>8</v>
+        <v>67</v>
       </c>
       <c r="D216" t="s">
         <v>21</v>
@@ -5061,26 +5067,49 @@
         <v>17</v>
       </c>
       <c r="G216" t="s">
-        <v>187</v>
+        <v>191</v>
+      </c>
+      <c r="H216" t="s">
+        <v>192</v>
       </c>
     </row>
     <row r="217" spans="1:12">
       <c r="A217" t="s">
-        <v>139</v>
+        <v>180</v>
       </c>
       <c r="B217" s="18">
-        <v>1.78</v>
+        <v>5.2499999999999998E-2</v>
       </c>
       <c r="C217" t="s">
         <v>8</v>
       </c>
       <c r="D217" t="s">
-        <v>66</v>
+        <v>21</v>
       </c>
       <c r="F217" t="s">
         <v>17</v>
       </c>
       <c r="G217" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="218" spans="1:12">
+      <c r="A218" t="s">
+        <v>139</v>
+      </c>
+      <c r="B218" s="18">
+        <v>1.78</v>
+      </c>
+      <c r="C218" t="s">
+        <v>8</v>
+      </c>
+      <c r="D218" t="s">
+        <v>66</v>
+      </c>
+      <c r="F218" t="s">
+        <v>17</v>
+      </c>
+      <c r="G218" t="s">
         <v>157</v>
       </c>
     </row>
@@ -5093,14 +5122,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CFFD7E1F-62C4-4B55-9EF4-FABFBE79AE8D}">
   <dimension ref="A1:L8"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:12">
       <c r="A1" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="3" spans="1:12" ht="15.6">
+    <row r="3" spans="1:12" ht="15.75">
       <c r="A3" s="3" t="s">
         <v>64</v>
       </c>
@@ -5120,7 +5149,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="4" spans="1:12" ht="15.6">
+    <row r="4" spans="1:12" ht="15.75">
       <c r="A4" s="3" t="s">
         <v>64</v>
       </c>
@@ -5145,7 +5174,7 @@
       <c r="K4" s="2"/>
       <c r="L4" s="2"/>
     </row>
-    <row r="5" spans="1:12" ht="15.6">
+    <row r="5" spans="1:12" ht="15.75">
       <c r="A5" s="3" t="s">
         <v>64</v>
       </c>
@@ -5218,7 +5247,7 @@
       <c r="K7" s="15"/>
       <c r="L7" s="15"/>
     </row>
-    <row r="8" spans="1:12" ht="15.6">
+    <row r="8" spans="1:12" ht="15.75">
       <c r="A8" s="3" t="s">
         <v>64</v>
       </c>
@@ -5249,16 +5278,16 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{64A8E48C-ECCC-42B7-B70A-16D5D4E493BD}">
   <dimension ref="A1:G34"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5546875" defaultRowHeight="13.8"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="11.5546875" style="7"/>
-    <col min="2" max="2" width="22.44140625" style="7" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.6640625" style="7" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="19.33203125" style="7" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="21.6640625" style="7" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="19.33203125" style="7" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="18.6640625" style="7" bestFit="1" customWidth="1"/>
-    <col min="9" max="16384" width="11.5546875" style="7"/>
+    <col min="1" max="1" width="11.5703125" style="7"/>
+    <col min="2" max="2" width="22.42578125" style="7" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.7109375" style="7" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="19.28515625" style="7" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="21.7109375" style="7" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="19.28515625" style="7" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="18.7109375" style="7" bestFit="1" customWidth="1"/>
+    <col min="9" max="16384" width="11.5703125" style="7"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
@@ -5388,7 +5417,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="14.4">
+    <row r="9" spans="1:7" ht="15">
       <c r="B9" s="7" t="s">
         <v>95</v>
       </c>

</xml_diff>

<commit_message>
downscaled ammonia cracking infrastructure
</commit_message>
<xml_diff>
--- a/premise/data/additional_inventories/lci-hydrogen-transport.xlsx
+++ b/premise/data/additional_inventories/lci-hydrogen-transport.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ac145674\coding_projects\premise_h2-distribution\premise\data\additional_inventories\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6CBAFE06-043C-4FF3-9C2D-B8E35A7EAB79}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1FFEF69-9C17-488D-A13D-3A454BD04D90}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8655" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8652" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="hydrogen-transport" sheetId="1" r:id="rId1"/>
@@ -519,9 +519,6 @@
     <t>chemical factory, organics</t>
   </si>
   <si>
-    <t>Used as the ammonia cracker facility, lifetime 50a, 28 t of NH3 cracked per day, 300d per year</t>
-  </si>
-  <si>
     <t>Used as proxy for liquid ammonia storage at the facility before cracking,  lifetime 50a, 28 t of NH3 cracked per day, 300d per year</t>
   </si>
   <si>
@@ -673,6 +670,9 @@
   </si>
   <si>
     <t>electricity needed for the processes and compression</t>
+  </si>
+  <si>
+    <t>Used as the ammonia cracker facility, lifetime 50a, 28 t of NH3 cracked per day, 300d per year, input scaled to a tenth of the size due to smaller scale</t>
   </si>
 </sst>
 </file>
@@ -1122,23 +1122,23 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:L218"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="82.7109375" customWidth="1"/>
-    <col min="2" max="2" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="82.6640625" customWidth="1"/>
+    <col min="2" max="2" width="9.88671875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="23" customWidth="1"/>
-    <col min="4" max="4" width="13.7109375" customWidth="1"/>
-    <col min="5" max="5" width="17.140625" customWidth="1"/>
-    <col min="6" max="6" width="16.140625" customWidth="1"/>
-    <col min="7" max="7" width="85.42578125" customWidth="1"/>
-    <col min="8" max="8" width="25.42578125" customWidth="1"/>
-    <col min="11" max="11" width="13.28515625" customWidth="1"/>
-    <col min="12" max="12" width="43.85546875" customWidth="1"/>
-    <col min="13" max="13" width="13.28515625" customWidth="1"/>
-    <col min="14" max="14" width="14.28515625" customWidth="1"/>
+    <col min="4" max="4" width="13.6640625" customWidth="1"/>
+    <col min="5" max="5" width="17.109375" customWidth="1"/>
+    <col min="6" max="6" width="16.109375" customWidth="1"/>
+    <col min="7" max="7" width="85.44140625" customWidth="1"/>
+    <col min="8" max="8" width="25.44140625" customWidth="1"/>
+    <col min="11" max="11" width="13.33203125" customWidth="1"/>
+    <col min="12" max="12" width="43.88671875" customWidth="1"/>
+    <col min="13" max="13" width="13.33203125" customWidth="1"/>
+    <col min="14" max="14" width="14.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="15.75">
+    <row r="1" spans="1:9" ht="15.6">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1146,7 +1146,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="15.75">
+    <row r="3" spans="1:9" ht="15.6">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
@@ -1208,7 +1208,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="15.75">
+    <row r="10" spans="1:9" ht="15.6">
       <c r="A10" s="1" t="s">
         <v>10</v>
       </c>
@@ -1264,7 +1264,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="13" spans="1:9" ht="15.75">
+    <row r="13" spans="1:9" ht="15.6">
       <c r="A13" s="3" t="s">
         <v>74</v>
       </c>
@@ -1311,7 +1311,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="15" spans="1:9" ht="15.75">
+    <row r="15" spans="1:9" ht="15.6">
       <c r="A15" s="3" t="s">
         <v>64</v>
       </c>
@@ -1356,7 +1356,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="18" spans="1:9" ht="15.75">
+    <row r="18" spans="1:9" ht="15.6">
       <c r="A18" s="1" t="s">
         <v>2</v>
       </c>
@@ -1418,7 +1418,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="25" spans="1:9" ht="15.75">
+    <row r="25" spans="1:9" ht="15.6">
       <c r="A25" s="1" t="s">
         <v>10</v>
       </c>
@@ -1474,7 +1474,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="28" spans="1:9" ht="15.75">
+    <row r="28" spans="1:9" ht="15.6">
       <c r="A28" s="3" t="s">
         <v>74</v>
       </c>
@@ -1521,7 +1521,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="30" spans="1:9" ht="15.75">
+    <row r="30" spans="1:9" ht="15.6">
       <c r="A30" s="3" t="s">
         <v>64</v>
       </c>
@@ -1566,12 +1566,12 @@
         <v>71</v>
       </c>
     </row>
-    <row r="33" spans="1:8" ht="15.75">
+    <row r="33" spans="1:8" ht="15.6">
       <c r="A33" s="4" t="s">
         <v>2</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="C33" s="5"/>
       <c r="D33" s="5"/>
@@ -1669,7 +1669,7 @@
         <v>14</v>
       </c>
       <c r="B40" s="12" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="C40" s="5"/>
       <c r="D40" s="5"/>
@@ -1692,7 +1692,7 @@
       <c r="G41" s="5"/>
       <c r="H41" s="5"/>
     </row>
-    <row r="42" spans="1:8" ht="15.75">
+    <row r="42" spans="1:8" ht="15.6">
       <c r="A42" s="4" t="s">
         <v>10</v>
       </c>
@@ -2155,12 +2155,12 @@
       </c>
       <c r="H61" s="5"/>
     </row>
-    <row r="63" spans="1:8" ht="15.75">
+    <row r="63" spans="1:8" ht="15.6">
       <c r="A63" s="4" t="s">
         <v>2</v>
       </c>
       <c r="B63" s="4" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="C63" s="5"/>
       <c r="D63" s="5"/>
@@ -2258,7 +2258,7 @@
         <v>14</v>
       </c>
       <c r="B70" s="12" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="C70" s="5"/>
       <c r="D70" s="5"/>
@@ -2281,7 +2281,7 @@
       <c r="G71" s="5"/>
       <c r="H71" s="5"/>
     </row>
-    <row r="72" spans="1:8" ht="15.75">
+    <row r="72" spans="1:8" ht="15.6">
       <c r="A72" s="4" t="s">
         <v>10</v>
       </c>
@@ -2386,7 +2386,7 @@
         <v>17</v>
       </c>
       <c r="G76" s="12" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="H76" s="5" t="s">
         <v>41</v>
@@ -2719,7 +2719,7 @@
         <v>6</v>
       </c>
       <c r="B92" s="15" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="C92" s="15"/>
       <c r="D92" s="15"/>
@@ -2737,7 +2737,7 @@
         <v>51</v>
       </c>
       <c r="B93" s="15" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="C93" s="15"/>
       <c r="D93" s="15"/>
@@ -2904,7 +2904,7 @@
       <c r="K100" s="15"/>
       <c r="L100" s="15"/>
     </row>
-    <row r="101" spans="1:12" ht="15.75">
+    <row r="101" spans="1:12" ht="15.6">
       <c r="A101" s="3" t="s">
         <v>64</v>
       </c>
@@ -3043,7 +3043,7 @@
         <v>6</v>
       </c>
       <c r="B107" s="15" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C107" s="15"/>
       <c r="D107" s="15"/>
@@ -3061,7 +3061,7 @@
         <v>51</v>
       </c>
       <c r="B108" s="15" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="C108" s="15"/>
       <c r="D108" s="15"/>
@@ -3375,7 +3375,7 @@
         <v>2</v>
       </c>
       <c r="B122" s="13" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="C122" s="15"/>
       <c r="D122" s="15"/>
@@ -3393,7 +3393,7 @@
         <v>6</v>
       </c>
       <c r="B123" s="15" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="C123" s="15"/>
       <c r="D123" s="15"/>
@@ -3411,7 +3411,7 @@
         <v>51</v>
       </c>
       <c r="B124" s="15" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="C124" s="15"/>
       <c r="D124" s="15"/>
@@ -3601,7 +3601,7 @@
         <v>157</v>
       </c>
       <c r="H132" s="15" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="I132" s="15"/>
       <c r="J132" s="15"/>
@@ -3610,7 +3610,7 @@
     </row>
     <row r="133" spans="1:12">
       <c r="A133" s="15" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B133" s="17">
         <v>3.4299999999999999E-9</v>
@@ -3626,17 +3626,17 @@
         <v>17</v>
       </c>
       <c r="G133" t="s">
+        <v>198</v>
+      </c>
+      <c r="H133" s="15" t="s">
         <v>199</v>
-      </c>
-      <c r="H133" s="15" t="s">
-        <v>200</v>
       </c>
       <c r="I133" s="15"/>
       <c r="J133" s="15"/>
       <c r="K133" s="15"/>
       <c r="L133" s="15"/>
     </row>
-    <row r="134" spans="1:12" ht="15.75">
+    <row r="134" spans="1:12" ht="15.6">
       <c r="A134" s="3" t="s">
         <v>64</v>
       </c>
@@ -3682,7 +3682,7 @@
       </c>
       <c r="G135" s="15"/>
       <c r="H135" s="15" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="I135" s="15"/>
       <c r="J135" s="15"/>
@@ -3726,7 +3726,7 @@
         <v>6</v>
       </c>
       <c r="B138" s="15" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="C138" s="15"/>
       <c r="D138" s="15"/>
@@ -3744,7 +3744,7 @@
         <v>51</v>
       </c>
       <c r="B139" s="15" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="C139" s="15"/>
       <c r="D139" s="15"/>
@@ -3939,7 +3939,7 @@
     </row>
     <row r="148" spans="1:12">
       <c r="A148" s="15" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B148" s="17">
         <v>3.4299999999999999E-9</v>
@@ -3955,10 +3955,10 @@
         <v>17</v>
       </c>
       <c r="G148" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="H148" s="15" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="I148" s="15"/>
       <c r="J148" s="15"/>
@@ -4134,7 +4134,7 @@
         <v>6</v>
       </c>
       <c r="B156" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="C156" s="15"/>
       <c r="D156" s="15"/>
@@ -4152,7 +4152,7 @@
         <v>51</v>
       </c>
       <c r="B157" s="15" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="C157" s="15"/>
       <c r="D157" s="15"/>
@@ -4343,7 +4343,7 @@
         <v>162</v>
       </c>
       <c r="H165" s="15" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="I165" s="15"/>
       <c r="J165" s="15"/>
@@ -4355,8 +4355,8 @@
         <v>163</v>
       </c>
       <c r="B166" s="17">
-        <f>1/(28*1000*300*50)</f>
-        <v>2.380952380952381E-9</v>
+        <f>1/(28*1000*300*50*10)</f>
+        <v>2.380952380952381E-10</v>
       </c>
       <c r="C166" s="15" t="s">
         <v>8</v>
@@ -4372,7 +4372,7 @@
         <v>164</v>
       </c>
       <c r="H166" s="15" t="s">
-        <v>165</v>
+        <v>216</v>
       </c>
       <c r="I166" s="15"/>
     </row>
@@ -4397,7 +4397,7 @@
         <v>62</v>
       </c>
       <c r="H167" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="169" spans="1:12">
@@ -4405,7 +4405,7 @@
         <v>2</v>
       </c>
       <c r="B169" s="13" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="170" spans="1:12">
@@ -4413,7 +4413,7 @@
         <v>6</v>
       </c>
       <c r="B170" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="171" spans="1:12">
@@ -4421,7 +4421,7 @@
         <v>51</v>
       </c>
       <c r="B171" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
     <row r="172" spans="1:12">
@@ -4429,7 +4429,7 @@
         <v>5</v>
       </c>
       <c r="B172" s="12" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
     </row>
     <row r="173" spans="1:12">
@@ -4518,15 +4518,15 @@
         <v>16</v>
       </c>
       <c r="G178" t="s">
+        <v>168</v>
+      </c>
+      <c r="H178" t="s">
         <v>169</v>
-      </c>
-      <c r="H178" t="s">
-        <v>170</v>
       </c>
     </row>
     <row r="179" spans="1:9">
       <c r="A179" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B179" s="18">
         <v>0.81499999999999995</v>
@@ -4541,7 +4541,7 @@
         <v>17</v>
       </c>
       <c r="G179" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="H179" t="s">
         <v>138</v>
@@ -4549,7 +4549,7 @@
     </row>
     <row r="180" spans="1:9">
       <c r="A180" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="B180" s="18">
         <v>5.1499999999999998E-5</v>
@@ -4564,7 +4564,7 @@
         <v>17</v>
       </c>
       <c r="G180" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="H180" t="s">
         <v>138</v>
@@ -4612,7 +4612,7 @@
     </row>
     <row r="183" spans="1:9">
       <c r="A183" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="B183" s="18">
         <v>5.1499999999999998E-5</v>
@@ -4627,7 +4627,7 @@
         <v>17</v>
       </c>
       <c r="G183" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="184" spans="1:9">
@@ -4737,7 +4737,7 @@
         <v>2</v>
       </c>
       <c r="B191" s="13" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="192" spans="1:9">
@@ -4745,7 +4745,7 @@
         <v>6</v>
       </c>
       <c r="B192" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="193" spans="1:12">
@@ -4753,7 +4753,7 @@
         <v>51</v>
       </c>
       <c r="B193" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
     </row>
     <row r="194" spans="1:12">
@@ -4761,7 +4761,7 @@
         <v>5</v>
       </c>
       <c r="B194" s="12" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
     </row>
     <row r="195" spans="1:12">
@@ -4777,7 +4777,7 @@
         <v>14</v>
       </c>
       <c r="B196" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="197" spans="1:12">
@@ -4833,7 +4833,7 @@
     </row>
     <row r="200" spans="1:12">
       <c r="A200" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B200" s="18">
         <v>1</v>
@@ -4848,15 +4848,15 @@
         <v>16</v>
       </c>
       <c r="G200" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="H200" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="201" spans="1:12">
       <c r="A201" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="B201" s="18">
         <v>4.4300000000000002E-10</v>
@@ -4871,7 +4871,7 @@
         <v>17</v>
       </c>
       <c r="G201" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
     </row>
     <row r="202" spans="1:12">
@@ -4913,7 +4913,7 @@
         <v>2</v>
       </c>
       <c r="B205" s="13" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="206" spans="1:12">
@@ -4921,7 +4921,7 @@
         <v>6</v>
       </c>
       <c r="B206" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="207" spans="1:12">
@@ -4929,7 +4929,7 @@
         <v>51</v>
       </c>
       <c r="B207" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="208" spans="1:12">
@@ -4937,7 +4937,7 @@
         <v>5</v>
       </c>
       <c r="B208" s="12" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
     </row>
     <row r="209" spans="1:12">
@@ -4953,7 +4953,7 @@
         <v>14</v>
       </c>
       <c r="B210" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="211" spans="1:12">
@@ -5009,7 +5009,7 @@
     </row>
     <row r="214" spans="1:12">
       <c r="A214" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="B214" s="18">
         <v>1</v>
@@ -5024,15 +5024,15 @@
         <v>16</v>
       </c>
       <c r="G214" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="H214" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="215" spans="1:12">
       <c r="A215" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="B215" s="18">
         <v>0.91700000000000004</v>
@@ -5047,12 +5047,12 @@
         <v>17</v>
       </c>
       <c r="G215" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="216" spans="1:12">
       <c r="A216" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B216" s="18">
         <v>0.03</v>
@@ -5067,15 +5067,15 @@
         <v>17</v>
       </c>
       <c r="G216" t="s">
+        <v>190</v>
+      </c>
+      <c r="H216" t="s">
         <v>191</v>
-      </c>
-      <c r="H216" t="s">
-        <v>192</v>
       </c>
     </row>
     <row r="217" spans="1:12">
       <c r="A217" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="B217" s="18">
         <v>5.2499999999999998E-2</v>
@@ -5090,7 +5090,7 @@
         <v>17</v>
       </c>
       <c r="G217" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
     </row>
     <row r="218" spans="1:12">
@@ -5122,14 +5122,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CFFD7E1F-62C4-4B55-9EF4-FABFBE79AE8D}">
   <dimension ref="A1:L8"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1" spans="1:12">
       <c r="A1" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="3" spans="1:12" ht="15.75">
+    <row r="3" spans="1:12" ht="15.6">
       <c r="A3" s="3" t="s">
         <v>64</v>
       </c>
@@ -5149,7 +5149,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="4" spans="1:12" ht="15.75">
+    <row r="4" spans="1:12" ht="15.6">
       <c r="A4" s="3" t="s">
         <v>64</v>
       </c>
@@ -5174,7 +5174,7 @@
       <c r="K4" s="2"/>
       <c r="L4" s="2"/>
     </row>
-    <row r="5" spans="1:12" ht="15.75">
+    <row r="5" spans="1:12" ht="15.6">
       <c r="A5" s="3" t="s">
         <v>64</v>
       </c>
@@ -5201,7 +5201,7 @@
     </row>
     <row r="6" spans="1:12">
       <c r="A6" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B6" s="18">
         <v>0.17599999999999999</v>
@@ -5216,7 +5216,7 @@
         <v>17</v>
       </c>
       <c r="G6" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="7" spans="1:12">
@@ -5247,7 +5247,7 @@
       <c r="K7" s="15"/>
       <c r="L7" s="15"/>
     </row>
-    <row r="8" spans="1:12" ht="15.75">
+    <row r="8" spans="1:12" ht="15.6">
       <c r="A8" s="3" t="s">
         <v>64</v>
       </c>
@@ -5267,7 +5267,7 @@
         <v>65</v>
       </c>
       <c r="H8" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
   </sheetData>
@@ -5278,16 +5278,16 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{64A8E48C-ECCC-42B7-B70A-16D5D4E493BD}">
   <dimension ref="A1:G34"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="14.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5546875" defaultRowHeight="13.8"/>
   <cols>
-    <col min="1" max="1" width="11.5703125" style="7"/>
-    <col min="2" max="2" width="22.42578125" style="7" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.7109375" style="7" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="19.28515625" style="7" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="21.7109375" style="7" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="19.28515625" style="7" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="18.7109375" style="7" bestFit="1" customWidth="1"/>
-    <col min="9" max="16384" width="11.5703125" style="7"/>
+    <col min="1" max="1" width="11.5546875" style="7"/>
+    <col min="2" max="2" width="22.44140625" style="7" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.6640625" style="7" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="19.33203125" style="7" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="21.6640625" style="7" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="19.33203125" style="7" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="18.6640625" style="7" bestFit="1" customWidth="1"/>
+    <col min="9" max="16384" width="11.5546875" style="7"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
@@ -5300,10 +5300,10 @@
         <v>125</v>
       </c>
       <c r="C2" s="7" t="s">
+        <v>213</v>
+      </c>
+      <c r="D2" s="7" t="s">
         <v>214</v>
-      </c>
-      <c r="D2" s="7" t="s">
-        <v>215</v>
       </c>
       <c r="E2" s="7" t="s">
         <v>83</v>
@@ -5417,7 +5417,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="15">
+    <row r="9" spans="1:7" ht="14.4">
       <c r="B9" s="7" t="s">
         <v>95</v>
       </c>

</xml_diff>

<commit_message>
changed h2 helping activities units from <unit> to <kilogram>
</commit_message>
<xml_diff>
--- a/premise/data/additional_inventories/lci-hydrogen-transport.xlsx
+++ b/premise/data/additional_inventories/lci-hydrogen-transport.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ac145674\coding_projects\premise_h2-distribution\premise\data\additional_inventories\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1FFEF69-9C17-488D-A13D-3A454BD04D90}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B90B4E6-B74C-4C2D-89BC-D2982588EC69}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8652" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8655" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="hydrogen-transport" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="926" uniqueCount="217">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="921" uniqueCount="217">
   <si>
     <t>Database</t>
   </si>
@@ -1122,23 +1122,23 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:L218"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="82.6640625" customWidth="1"/>
-    <col min="2" max="2" width="9.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="82.7109375" customWidth="1"/>
+    <col min="2" max="2" width="9.85546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="23" customWidth="1"/>
-    <col min="4" max="4" width="13.6640625" customWidth="1"/>
-    <col min="5" max="5" width="17.109375" customWidth="1"/>
-    <col min="6" max="6" width="16.109375" customWidth="1"/>
-    <col min="7" max="7" width="85.44140625" customWidth="1"/>
-    <col min="8" max="8" width="25.44140625" customWidth="1"/>
-    <col min="11" max="11" width="13.33203125" customWidth="1"/>
-    <col min="12" max="12" width="43.88671875" customWidth="1"/>
-    <col min="13" max="13" width="13.33203125" customWidth="1"/>
-    <col min="14" max="14" width="14.33203125" customWidth="1"/>
+    <col min="4" max="4" width="13.7109375" customWidth="1"/>
+    <col min="5" max="5" width="17.140625" customWidth="1"/>
+    <col min="6" max="6" width="16.140625" customWidth="1"/>
+    <col min="7" max="7" width="85.42578125" customWidth="1"/>
+    <col min="8" max="8" width="25.42578125" customWidth="1"/>
+    <col min="11" max="11" width="13.28515625" customWidth="1"/>
+    <col min="12" max="12" width="43.85546875" customWidth="1"/>
+    <col min="13" max="13" width="13.28515625" customWidth="1"/>
+    <col min="14" max="14" width="14.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="15.6">
+    <row r="1" spans="1:9" ht="15.75">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1146,7 +1146,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="15.6">
+    <row r="3" spans="1:9" ht="15.75">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
@@ -1208,7 +1208,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="15.6">
+    <row r="10" spans="1:9" ht="15.75">
       <c r="A10" s="1" t="s">
         <v>10</v>
       </c>
@@ -1264,7 +1264,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="13" spans="1:9" ht="15.6">
+    <row r="13" spans="1:9" ht="15.75">
       <c r="A13" s="3" t="s">
         <v>74</v>
       </c>
@@ -1311,7 +1311,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="15" spans="1:9" ht="15.6">
+    <row r="15" spans="1:9" ht="15.75">
       <c r="A15" s="3" t="s">
         <v>64</v>
       </c>
@@ -1356,7 +1356,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="18" spans="1:9" ht="15.6">
+    <row r="18" spans="1:9" ht="15.75">
       <c r="A18" s="1" t="s">
         <v>2</v>
       </c>
@@ -1418,7 +1418,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="25" spans="1:9" ht="15.6">
+    <row r="25" spans="1:9" ht="15.75">
       <c r="A25" s="1" t="s">
         <v>10</v>
       </c>
@@ -1474,7 +1474,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="28" spans="1:9" ht="15.6">
+    <row r="28" spans="1:9" ht="15.75">
       <c r="A28" s="3" t="s">
         <v>74</v>
       </c>
@@ -1521,7 +1521,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="30" spans="1:9" ht="15.6">
+    <row r="30" spans="1:9" ht="15.75">
       <c r="A30" s="3" t="s">
         <v>64</v>
       </c>
@@ -1566,7 +1566,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="33" spans="1:8" ht="15.6">
+    <row r="33" spans="1:8" ht="15.75">
       <c r="A33" s="4" t="s">
         <v>2</v>
       </c>
@@ -1692,7 +1692,7 @@
       <c r="G41" s="5"/>
       <c r="H41" s="5"/>
     </row>
-    <row r="42" spans="1:8" ht="15.6">
+    <row r="42" spans="1:8" ht="15.75">
       <c r="A42" s="4" t="s">
         <v>10</v>
       </c>
@@ -2155,7 +2155,7 @@
       </c>
       <c r="H61" s="5"/>
     </row>
-    <row r="63" spans="1:8" ht="15.6">
+    <row r="63" spans="1:8" ht="15.75">
       <c r="A63" s="4" t="s">
         <v>2</v>
       </c>
@@ -2281,7 +2281,7 @@
       <c r="G71" s="5"/>
       <c r="H71" s="5"/>
     </row>
-    <row r="72" spans="1:8" ht="15.6">
+    <row r="72" spans="1:8" ht="15.75">
       <c r="A72" s="4" t="s">
         <v>10</v>
       </c>
@@ -2809,7 +2809,7 @@
         <v>13</v>
       </c>
       <c r="B97" s="15" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="C97" s="15"/>
       <c r="D97" s="15"/>
@@ -2886,8 +2886,9 @@
       <c r="C100" s="15" t="s">
         <v>8</v>
       </c>
-      <c r="D100" s="15" t="s">
-        <v>13</v>
+      <c r="D100" s="15" t="str">
+        <f>B97</f>
+        <v>kilogram</v>
       </c>
       <c r="E100" s="15"/>
       <c r="F100" s="15" t="s">
@@ -2904,7 +2905,7 @@
       <c r="K100" s="15"/>
       <c r="L100" s="15"/>
     </row>
-    <row r="101" spans="1:12" ht="15.6">
+    <row r="101" spans="1:12" ht="15.75">
       <c r="A101" s="3" t="s">
         <v>64</v>
       </c>
@@ -3484,7 +3485,7 @@
         <v>13</v>
       </c>
       <c r="B128" s="15" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="C128" s="15"/>
       <c r="D128" s="15"/>
@@ -3562,8 +3563,9 @@
       <c r="C131" s="15" t="s">
         <v>8</v>
       </c>
-      <c r="D131" s="15" t="s">
-        <v>13</v>
+      <c r="D131" s="15" t="str">
+        <f>B128</f>
+        <v>kilogram</v>
       </c>
       <c r="E131" s="15"/>
       <c r="F131" s="15" t="s">
@@ -3636,7 +3638,7 @@
       <c r="K133" s="15"/>
       <c r="L133" s="15"/>
     </row>
-    <row r="134" spans="1:12" ht="15.6">
+    <row r="134" spans="1:12" ht="15.75">
       <c r="A134" s="3" t="s">
         <v>64</v>
       </c>
@@ -3816,7 +3818,7 @@
         <v>13</v>
       </c>
       <c r="B143" s="15" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="C143" s="15"/>
       <c r="D143" s="15"/>
@@ -3894,8 +3896,9 @@
       <c r="C146" s="15" t="s">
         <v>8</v>
       </c>
-      <c r="D146" s="15" t="s">
-        <v>13</v>
+      <c r="D146" s="15" t="str">
+        <f>B143</f>
+        <v>kilogram</v>
       </c>
       <c r="E146" s="15"/>
       <c r="F146" s="15" t="s">
@@ -4224,7 +4227,7 @@
         <v>13</v>
       </c>
       <c r="B161" s="15" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="C161" s="15"/>
       <c r="D161" s="15"/>
@@ -4302,8 +4305,9 @@
       <c r="C164" s="15" t="s">
         <v>8</v>
       </c>
-      <c r="D164" s="15" t="s">
-        <v>13</v>
+      <c r="D164" s="15" t="str">
+        <f>B161</f>
+        <v>kilogram</v>
       </c>
       <c r="E164" s="15"/>
       <c r="F164" s="15" t="s">
@@ -4454,7 +4458,7 @@
         <v>13</v>
       </c>
       <c r="B175" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
     </row>
     <row r="176" spans="1:12">
@@ -4511,8 +4515,9 @@
       <c r="C178" t="s">
         <v>8</v>
       </c>
-      <c r="D178" t="s">
-        <v>13</v>
+      <c r="D178" t="str">
+        <f>B175</f>
+        <v>kilogram</v>
       </c>
       <c r="F178" t="s">
         <v>16</v>
@@ -5122,14 +5127,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CFFD7E1F-62C4-4B55-9EF4-FABFBE79AE8D}">
   <dimension ref="A1:L8"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:12">
       <c r="A1" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="3" spans="1:12" ht="15.6">
+    <row r="3" spans="1:12" ht="15.75">
       <c r="A3" s="3" t="s">
         <v>64</v>
       </c>
@@ -5149,7 +5154,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="4" spans="1:12" ht="15.6">
+    <row r="4" spans="1:12" ht="15.75">
       <c r="A4" s="3" t="s">
         <v>64</v>
       </c>
@@ -5174,7 +5179,7 @@
       <c r="K4" s="2"/>
       <c r="L4" s="2"/>
     </row>
-    <row r="5" spans="1:12" ht="15.6">
+    <row r="5" spans="1:12" ht="15.75">
       <c r="A5" s="3" t="s">
         <v>64</v>
       </c>
@@ -5247,7 +5252,7 @@
       <c r="K7" s="15"/>
       <c r="L7" s="15"/>
     </row>
-    <row r="8" spans="1:12" ht="15.6">
+    <row r="8" spans="1:12" ht="15.75">
       <c r="A8" s="3" t="s">
         <v>64</v>
       </c>
@@ -5278,16 +5283,16 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{64A8E48C-ECCC-42B7-B70A-16D5D4E493BD}">
   <dimension ref="A1:G34"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5546875" defaultRowHeight="13.8"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="11.5546875" style="7"/>
-    <col min="2" max="2" width="22.44140625" style="7" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.6640625" style="7" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="19.33203125" style="7" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="21.6640625" style="7" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="19.33203125" style="7" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="18.6640625" style="7" bestFit="1" customWidth="1"/>
-    <col min="9" max="16384" width="11.5546875" style="7"/>
+    <col min="1" max="1" width="11.5703125" style="7"/>
+    <col min="2" max="2" width="22.42578125" style="7" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.7109375" style="7" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="19.28515625" style="7" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="21.7109375" style="7" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="19.28515625" style="7" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="18.7109375" style="7" bestFit="1" customWidth="1"/>
+    <col min="9" max="16384" width="11.5703125" style="7"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
@@ -5417,7 +5422,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="14.4">
+    <row r="9" spans="1:7" ht="15">
       <c r="B9" s="7" t="s">
         <v>95</v>
       </c>

</xml_diff>

<commit_message>
adjusted LHV of MDO fuel in lci
</commit_message>
<xml_diff>
--- a/premise/data/additional_inventories/lci-hydrogen-transport.xlsx
+++ b/premise/data/additional_inventories/lci-hydrogen-transport.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ac145674\coding_projects\premise_h2-distribution\premise\data\additional_inventories\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B90B4E6-B74C-4C2D-89BC-D2982588EC69}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA25538F-5D11-4668-A158-6CA8E0CD94C5}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8655" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1906,7 +1906,7 @@
       </c>
       <c r="B51" s="5">
         <f>(parameters!D10*parameters!D6/1000)*parameters!D9</f>
-        <v>1.4850480349344979E-4</v>
+        <v>1.4850480349344981E-5</v>
       </c>
       <c r="C51" s="12" t="s">
         <v>131</v>
@@ -1931,7 +1931,7 @@
       </c>
       <c r="B52" s="5">
         <f>((parameters!D15*parameters!D6/1000)*parameters!D9)+((parameters!D16*parameters!D6/1000)*(1-parameters!D9))</f>
-        <v>4.7617641921397384E-4</v>
+        <v>4.761764192139738E-5</v>
       </c>
       <c r="C52" s="5"/>
       <c r="D52" s="5" t="s">
@@ -2000,7 +2000,7 @@
       </c>
       <c r="B55" s="5">
         <f>((parameters!D6*parameters!D12/1000)*parameters!D9)+((parameters!D6*parameters!D13/1000)*(1-parameters!D9))+((parameters!D8/1000)*parameters!D23)</f>
-        <v>1.2346794829694324E-4</v>
+        <v>1.2363930829694324E-5</v>
       </c>
       <c r="C55" s="5"/>
       <c r="D55" s="5" t="s">
@@ -2069,7 +2069,7 @@
       </c>
       <c r="B58" s="5">
         <f>((parameters!D6*parameters!D17/1000)*parameters!D9)+((parameters!D6*parameters!D18/1000)*(1-parameters!D9))+((parameters!D8/1000*parameters!D27)*(parameters!D9))+((parameters!D8/1000)*parameters!D28)*(1-parameters!D9)</f>
-        <v>1.5558654148471616E-3</v>
+        <v>1.723990131004367E-4</v>
       </c>
       <c r="C58" s="5"/>
       <c r="D58" s="5" t="s">
@@ -2470,7 +2470,7 @@
       </c>
       <c r="B80" s="14">
         <f>(parameters!C10*parameters!C6/1000)*parameters!C9</f>
-        <v>6.4616593886462886E-6</v>
+        <v>1.4850480349344981E-5</v>
       </c>
       <c r="C80" s="12" t="s">
         <v>131</v>
@@ -2495,7 +2495,7 @@
       </c>
       <c r="B81" s="14">
         <f>(parameters!C22/1000)*(parameters!C8+parameters!C6)</f>
-        <v>3.1887360000000002E-3</v>
+        <v>6.875712E-3</v>
       </c>
       <c r="C81" s="5"/>
       <c r="D81" s="5" t="s">
@@ -2518,7 +2518,7 @@
       </c>
       <c r="B82" s="14">
         <f>(parameters!C24/1000)*(parameters!C8+parameters!C6)</f>
-        <v>2.5600000000000001E-6</v>
+        <v>5.5200000000000005E-6</v>
       </c>
       <c r="C82" s="5"/>
       <c r="D82" s="5" t="s">
@@ -2541,7 +2541,7 @@
       </c>
       <c r="B83" s="14">
         <f>(((parameters!C6+parameters!C8)/1000)*parameters!C23)</f>
-        <v>1.7408000000000001E-7</v>
+        <v>3.7535999999999999E-7</v>
       </c>
       <c r="C83" s="5"/>
       <c r="D83" s="5" t="s">
@@ -2564,7 +2564,7 @@
       </c>
       <c r="B84" s="14">
         <f>((parameters!C6+parameters!C8)/1000)*parameters!C25</f>
-        <v>1.2800000000000001E-7</v>
+        <v>2.7599999999999998E-7</v>
       </c>
       <c r="C84" s="5"/>
       <c r="D84" s="5" t="s">
@@ -2587,7 +2587,7 @@
       </c>
       <c r="B85" s="14">
         <f>parameters!C32*(parameters!C8+parameters!C6)/1000</f>
-        <v>1.28E-6</v>
+        <v>2.7600000000000003E-6</v>
       </c>
       <c r="C85" s="5"/>
       <c r="D85" s="5" t="s">
@@ -2610,7 +2610,7 @@
       </c>
       <c r="B86" s="14">
         <f>(((parameters!C8+parameters!C6)/1000)*parameters!C27)*(parameters!C9)+(((parameters!C8+parameters!C6)/1000)*parameters!C28)*(1-parameters!C9)</f>
-        <v>1.7079336244541486E-4</v>
+        <v>3.6827318777292575E-4</v>
       </c>
       <c r="C86" s="5"/>
       <c r="D86" s="5" t="s">
@@ -5325,7 +5325,7 @@
         <v>85</v>
       </c>
       <c r="C3" s="7">
-        <v>42.7</v>
+        <v>11.861000000000001</v>
       </c>
       <c r="D3" s="7">
         <v>5.1669999999999998</v>
@@ -5341,11 +5341,11 @@
       <c r="B4" s="7" t="s">
         <v>88</v>
       </c>
-      <c r="C4" s="7">
-        <v>2.75E-2</v>
+      <c r="C4" s="8">
+        <v>2.615E-2</v>
       </c>
       <c r="D4" s="8">
-        <v>2.75E-2</v>
+        <v>2.615E-2</v>
       </c>
       <c r="F4" s="7" t="s">
         <v>123</v>
@@ -5376,10 +5376,10 @@
         <v>92</v>
       </c>
       <c r="C6" s="7">
-        <v>1.14E-2</v>
+        <v>2.6200000000000001E-2</v>
       </c>
       <c r="D6" s="8">
-        <v>0.26200000000000001</v>
+        <v>2.6200000000000001E-2</v>
       </c>
       <c r="F6" s="7" t="s">
         <v>123</v>

</xml_diff>